<commit_message>
exclude non-wb countries from the scorecard variables
</commit_message>
<xml_diff>
--- a/data-raw/input/csc/csc_variables.xlsx
+++ b/data-raw/input/csc/csc_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/iedochie_worldbank_org/Documents/Documents/GitProjects/cliaretl/data-raw/input/csc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wb438023\github\cliaretl\data-raw\input\csc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{0E6CB0F2-6129-4144-BE56-08CC15B14098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43A2B1D2-3DF3-440E-A21D-35EE61A6025A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685AB6C3-A7CE-40AE-9208-BAE3DEA3C2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="71">
   <si>
     <t>Beneficiaries of social safety net programs</t>
   </si>
@@ -167,15 +167,6 @@
     <t>WB_CSC_EG_ELC_ACCS_ZS</t>
   </si>
   <si>
-    <t>GW of renewable energy capacity enabled</t>
-  </si>
-  <si>
-    <t>Renewable natural capital index</t>
-  </si>
-  <si>
-    <t>WB_CSC_ER_NCA_RNEW</t>
-  </si>
-  <si>
     <t>People using broadband internet as a percentage of the population</t>
   </si>
   <si>
@@ -219,12 +210,6 @@
   </si>
   <si>
     <t>WB_CSC_FX_OWN_TOTL_ZS</t>
-  </si>
-  <si>
-    <t>People &amp; businesses using financial services — Female (% of the female population)</t>
-  </si>
-  <si>
-    <t>Account ownership at a financial institution — female (%)</t>
   </si>
   <si>
     <t xml:space="preserve">More and better-paid jobs </t>
@@ -640,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="57.125" bestFit="1" customWidth="1"/>
@@ -651,16 +636,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -954,49 +939,21 @@
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s">
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
         <v>66</v>
-      </c>
-      <c r="B24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>69</v>
-      </c>
-      <c r="B25" t="s">
-        <v>70</v>
-      </c>
-      <c r="C25" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" t="s">
-        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1006,7 +963,7 @@
     <oddFooter>&amp;R_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Official Use Only</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="A2:D4 A5:D9 A24:D25 B12:D12 B11:D11 B10:D10 B13:D13 B14:D14 B15:D15 C16:D16 B17:D17 B18:D18 B19:D19 B20:D20 B21:D21 B22:D22 B23:D23" numberStoredAsText="1"/>
+    <ignoredError sqref="A2:D4 A5:D9 A22:D23 B12:D12 B11:D11 B10:D10 B13:D13 B14:D14 B15:D15 B16:D16 B17:D17 B18:D18 B19:D19 B20:D20 B21:D21" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>